<commit_message>
more on the checklist
</commit_message>
<xml_diff>
--- a/dspackagefolder/template/checklist/ML_CHECKLIST.xlsx
+++ b/dspackagefolder/template/checklist/ML_CHECKLIST.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajim\Desktop\NonPHD_Muizdeen\INTERVIEWS\dspackage\dspackagefolder\template\checklist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D84E5F-DE2E-4604-AEEC-9966C12DD531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1E0B36-800F-44AB-9CAF-A55047955176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>WHAT TO CHECK</t>
   </si>
@@ -121,6 +121,12 @@
   </si>
   <si>
     <t>A process is in place to update or retrain the model when necessary.</t>
+  </si>
+  <si>
+    <t>You have logged the count of the following:
+1. the rows of data
+2. the number of each class
+3. the number of missing rows for each column</t>
   </si>
 </sst>
 </file>
@@ -545,6 +551,11 @@
         <v>16</v>
       </c>
     </row>
+    <row r="17" spans="1:1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>17</v>

</xml_diff>